<commit_message>
identification of an error ca7a3d064090c3db07fb57114353c60de26ca3c1
</commit_message>
<xml_diff>
--- a/ig/update-vs-url/ValueSet-fr-core-organization-uf-activity-field.xlsx
+++ b/ig/update-vs-url/ValueSet-fr-core-organization-uf-activity-field.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
-    <sheet name="Include from fr-v2-3311" r:id="rId4" sheetId="2"/>
+    <sheet name="Include from FR Core CodeSyst" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-07T10:39:28+00:00</t>
+    <t>2023-11-07T10:47:16+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -141,7 +141,7 @@
     <t>System URI</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/CodeSystem/fr-v2-3311</t>
+    <t>https://hl7.fr/ig/fhir/core/CodeSystem/fr-core-v2-3311</t>
   </si>
 </sst>
 </file>

</xml_diff>